<commit_message>
Update docs: integrācijas, ieviešanas process, prezentācija, izplatītāji, demo
</commit_message>
<xml_diff>
--- a/docs/HOR integrācijas.xlsx
+++ b/docs/HOR integrācijas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Raivis.Biskaps\Documents\Claude\Projects\Horizon pārdošana\docs-qa\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://vitcazure-my.sharepoint.com/personal/raivis_biskaps_visma_com/Documents/Documents/Claude/Projects/Horizon pārdošana/docs-qa/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C49B02D5-1088-4A3F-9A26-2FE65FB9844B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{CED7D905-8F73-4A4A-A265-D1A0BD520F2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9834539D-23B1-4FA0-8375-C36B099DDE43}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="768" yWindow="768" windowWidth="21600" windowHeight="12396" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="integrācijas" sheetId="1" r:id="rId1"/>
@@ -280,13 +280,13 @@
     <t>Integrācijas apraksts</t>
   </si>
   <si>
-    <t>Links uz partnera lapu</t>
-  </si>
-  <si>
-    <t>Integrācijas partneris</t>
-  </si>
-  <si>
     <t>Kategorija</t>
+  </si>
+  <si>
+    <t>Integrācijas izstrādātājs</t>
+  </si>
+  <si>
+    <t>Links uz risinājuma lapu</t>
   </si>
 </sst>
 </file>
@@ -585,18 +585,19 @@
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="23.77734375" customWidth="1"/>
+    <col min="3" max="3" width="21.5546875" customWidth="1"/>
     <col min="4" max="4" width="369.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>86</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>84</v>

</xml_diff>